<commit_message>
Dashboard update 2026-07-31 23:37
</commit_message>
<xml_diff>
--- a/excel/Profitus.xlsx
+++ b/excel/Profitus.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Investavimas 2026.06.03\Profitus\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\evald\OneDrive\Dokumentai\portfolio-analytics\portfolio-dashboard-clean\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB36775F-E26F-4D33-BD71-CBE6747D04AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{838B28A5-FAED-4A9D-BA46-4EBB1B385605}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="13" activeTab="20" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -2710,7 +2710,7 @@
       </c>
       <c r="X3" s="13">
         <f ca="1">XIRR(Pinigai!K2:K200,Pinigai!A2:A200)</f>
-        <v>8.4797057509422305E-2</v>
+        <v>8.4387615323066725E-2</v>
       </c>
       <c r="AC3" s="10" t="str">
         <f ca="1">'Ocean 11 South, II'!AA2</f>
@@ -3211,7 +3211,7 @@
       </c>
       <c r="J12" s="10">
         <f ca="1">'Dvibutis Upelio g., Vilniaus r.'!B13</f>
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="K12" s="10" t="str">
         <f ca="1">'Dvibutis Upelio g., Vilniaus r.'!S3</f>
@@ -3268,7 +3268,7 @@
       </c>
       <c r="J13" s="10">
         <f ca="1">'Piekrasta Rezidence, Ryga XII'!B13</f>
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="K13" s="10" t="str">
         <f ca="1">'Piekrasta Rezidence, Ryga XII'!S3</f>
@@ -3325,7 +3325,7 @@
       </c>
       <c r="J14" s="10">
         <f ca="1">'Dvibutis Didžiojoje Riešėje'!B13</f>
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="K14" s="10" t="str">
         <f ca="1">'Dvibutis Didžiojoje Riešėje'!S3</f>
@@ -3382,7 +3382,7 @@
       </c>
       <c r="J15" s="10">
         <f ca="1">'Sklypas Kalnėnuose, Vilnius II'!B13</f>
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="K15" s="10" t="str">
         <f ca="1">'Sklypas Kalnėnuose, Vilnius II'!S3</f>
@@ -3439,7 +3439,7 @@
       </c>
       <c r="J16" s="10">
         <f ca="1">'Golf Hills Vilos, Alikantė'!B13</f>
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="K16" s="10" t="str">
         <f ca="1">'Golf Hills Vilos, Alikantė'!S3</f>
@@ -3496,7 +3496,7 @@
       </c>
       <c r="J17" s="10">
         <f ca="1">'Svajonių Daugiabutis, Kaunas'!B13</f>
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="K17" s="10" t="str">
         <f ca="1">'Svajonių Daugiabutis, Kaunas'!S3</f>
@@ -3552,7 +3552,7 @@
       </c>
       <c r="J18" s="10">
         <f ca="1">'Brivibas 28, Jūrmala'!B13</f>
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="K18" s="10" t="str">
         <f ca="1">'Brivibas 28, Jūrmala'!S3</f>
@@ -3609,7 +3609,7 @@
       </c>
       <c r="J19" s="10">
         <f ca="1">'Europos 70, Kaunas XX'!B13</f>
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="K19" s="10" t="str">
         <f ca="1">'Europos 70, Kaunas XX'!S3</f>
@@ -3666,7 +3666,7 @@
       </c>
       <c r="J20" s="10">
         <f ca="1">'Molėtų Oazė XII'!B13</f>
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="K20" s="10" t="str">
         <f ca="1">'Molėtų Oazė XII'!S3</f>
@@ -3723,7 +3723,7 @@
       </c>
       <c r="J21" s="10">
         <f ca="1">'Dvibučių kvartalas Kauno r. II'!B13</f>
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="K21" s="10" t="str">
         <f ca="1">'Dvibučių kvartalas Kauno r. II'!S3</f>
@@ -4351,7 +4351,7 @@
       </c>
       <c r="B13" s="10">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D13" s="19"/>
       <c r="E13" s="5"/>
@@ -5505,7 +5505,7 @@
       </c>
       <c r="B13" s="10">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D13" s="19"/>
       <c r="E13" s="5"/>
@@ -6659,7 +6659,7 @@
       </c>
       <c r="B13" s="10">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D13" s="19"/>
       <c r="E13" s="5"/>
@@ -15601,7 +15601,7 @@
       </c>
       <c r="L1" s="13">
         <f ca="1">XIRR(K2:K200,A2:A200)</f>
-        <v>8.4797057509422305E-2</v>
+        <v>8.4387615323066725E-2</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
@@ -17133,7 +17133,7 @@
     <row r="200" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A200" s="23">
         <f ca="1">TODAY()</f>
-        <v>46232</v>
+        <v>46234</v>
       </c>
       <c r="B200" s="2"/>
       <c r="C200" s="2"/>
@@ -19931,7 +19931,7 @@
       </c>
       <c r="B13" s="10">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="D13" s="11"/>
       <c r="E13" s="5"/>
@@ -21061,7 +21061,7 @@
       </c>
       <c r="B13" s="10">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="D13" s="11"/>
       <c r="E13" s="5"/>
@@ -22191,7 +22191,7 @@
       </c>
       <c r="B13" s="10">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="D13" s="11"/>
       <c r="E13" s="5"/>
@@ -23387,7 +23387,7 @@
       </c>
       <c r="B13" s="10">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="D13" s="11">
         <v>46470</v>
@@ -24530,7 +24530,7 @@
       </c>
       <c r="B13" s="10">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="D13" s="19"/>
       <c r="E13" s="5"/>
@@ -25668,7 +25668,7 @@
       </c>
       <c r="B13" s="10">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="D13" s="19"/>
       <c r="E13" s="5"/>
@@ -26806,7 +26806,7 @@
       </c>
       <c r="B13" s="10">
         <f ca="1">IF(B11&lt;&gt;N3,(TODAY()-B12)*-1,"")</f>
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="D13" s="19"/>
       <c r="E13" s="5"/>

</xml_diff>